<commit_message>
User Access Maintenance FRS v1.3 aligned with BIBS: Identity Synchronisation, Session Timed Out and Audit Trail screens, updated Login, inactivity warning, Users and Separation of Duties, every screenshot taken again, settings for the points BDOI decides, identity notices, integrations and test cases
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_Inputs_BRD-11_Business_Unit_Requirements_Collection_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_Inputs_BRD-11_Business_Unit_Requirements_Collection_v1.0.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Start here'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Documents and print formats'!$A$12:$K$23</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Documents and print formats'!$12:$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'E-mail wordings'!$A$12:$K$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'E-mail wordings'!$A$12:$K$36</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'E-mail wordings'!$12:$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Schedules and timings'!$A$12:$K$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Schedules and timings'!$12:$12</definedName>
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="D23" s="14" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="24">
@@ -7455,7 +7455,7 @@
       </c>
       <c r="C6" s="24" t="inlineStr">
         <is>
-          <t>21 items</t>
+          <t>23 items</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
@@ -7469,7 +7469,7 @@
         </is>
       </c>
       <c r="F6" s="24" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G6" s="24">
         <f>COUNTIF('E-mail wordings'!K:K,"Open")</f>
@@ -8845,7 +8845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10333,47 +10333,47 @@
     <row r="34">
       <c r="A34" s="22" t="inlineStr">
         <is>
-          <t>RC-EML-21</t>
+          <t>NT-21</t>
         </is>
       </c>
       <c r="B34" s="22" t="inlineStr">
         <is>
-          <t>Sender and footer of the e-mails</t>
+          <t>Identity event to review</t>
         </is>
       </c>
       <c r="C34" s="22" t="inlineStr">
         <is>
-          <t>BRD NFR p.17 (10)</t>
+          <t>BRD 1.001 (user enrolment); BRD NFR p.13 (1)</t>
         </is>
       </c>
       <c r="D34" s="22" t="inlineStr">
         <is>
-          <t>Annex T</t>
+          <t>Annex T; FRUM.002.02, FRUM.003.03</t>
         </is>
       </c>
       <c r="E34" s="22" t="inlineStr">
         <is>
-          <t>The sender address of each environment and, if required, the standard footer or disclaimer of BDOI e-mails.</t>
+          <t>Approve the wording, the trigger and the recipients. Subject: Identity event &lt;event no&gt; needs review. Text: &lt;UIDM-ISC | Enterprise SSO&gt; event &lt;Joiner | Mover | Leaver | Rehire | Status&gt; of Windows ID &lt;Windows ID&gt; was &lt;refused | failed&gt;: &lt;reason&gt;</t>
         </is>
       </c>
       <c r="F34" s="22" t="inlineStr">
         <is>
-          <t>Address per environment; footer text</t>
+          <t>Approve, or the new wording</t>
         </is>
       </c>
       <c r="G34" s="22" t="inlineStr">
         <is>
-          <t>bibs-noreply@ (domain of BDOI)</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="H34" s="22" t="inlineStr">
         <is>
-          <t>BDOI IT</t>
+          <t>Process Owner (Business Administration)</t>
         </is>
       </c>
       <c r="I34" s="22" t="inlineStr">
         <is>
-          <t>16-Jul-2027</t>
+          <t>01-Dec-2026</t>
         </is>
       </c>
       <c r="J34" s="22" t="inlineStr"/>
@@ -10383,8 +10383,114 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="24" t="inlineStr">
+        <is>
+          <t>NT-22</t>
+        </is>
+      </c>
+      <c r="B35" s="24" t="inlineStr">
+        <is>
+          <t>Break-glass sign-in</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>BRD NFR p.17 (1)</t>
+        </is>
+      </c>
+      <c r="D35" s="24" t="inlineStr">
+        <is>
+          <t>Annex T; FRUM.001.06</t>
+        </is>
+      </c>
+      <c r="E35" s="24" t="inlineStr">
+        <is>
+          <t>Approve the wording, the trigger and the recipients. Subject: Break-glass sign-in. Text: Break-glass administrator &lt;name&gt; (&lt;user ID&gt;) signed in with a local password at &lt;dd-MMM-yyyy HH:mm&gt; from &lt;address&gt;. Review the use within one working day.</t>
+        </is>
+      </c>
+      <c r="F35" s="24" t="inlineStr">
+        <is>
+          <t>Approve, or the new wording</t>
+        </is>
+      </c>
+      <c r="G35" s="24" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H35" s="24" t="inlineStr">
+        <is>
+          <t>Process Owner (Business Administration)</t>
+        </is>
+      </c>
+      <c r="I35" s="24" t="inlineStr">
+        <is>
+          <t>01-Dec-2026</t>
+        </is>
+      </c>
+      <c r="J35" s="24" t="inlineStr"/>
+      <c r="K35" s="24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="inlineStr">
+        <is>
+          <t>RC-EML-21</t>
+        </is>
+      </c>
+      <c r="B36" s="22" t="inlineStr">
+        <is>
+          <t>Sender and footer of the e-mails</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="inlineStr">
+        <is>
+          <t>BRD NFR p.17 (10)</t>
+        </is>
+      </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>Annex T</t>
+        </is>
+      </c>
+      <c r="E36" s="22" t="inlineStr">
+        <is>
+          <t>The sender address of each environment and, if required, the standard footer or disclaimer of BDOI e-mails.</t>
+        </is>
+      </c>
+      <c r="F36" s="22" t="inlineStr">
+        <is>
+          <t>Address per environment; footer text</t>
+        </is>
+      </c>
+      <c r="G36" s="22" t="inlineStr">
+        <is>
+          <t>bibs-noreply@ (domain of BDOI)</t>
+        </is>
+      </c>
+      <c r="H36" s="22" t="inlineStr">
+        <is>
+          <t>BDOI IT</t>
+        </is>
+      </c>
+      <c r="I36" s="22" t="inlineStr">
+        <is>
+          <t>16-Jul-2027</t>
+        </is>
+      </c>
+      <c r="J36" s="22" t="inlineStr"/>
+      <c r="K36" s="22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A12:K34"/>
+  <autoFilter ref="A12:K36"/>
   <mergeCells count="5">
     <mergeCell ref="B4:K4"/>
     <mergeCell ref="B6:K6"/>
@@ -10393,7 +10499,7 @@
     <mergeCell ref="B5:K5"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K14:K334" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="K14:K336" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$B$2:$B$4</formula1>
     </dataValidation>
   </dataValidations>
@@ -12278,7 +12384,7 @@
       </c>
       <c r="E21" s="24" t="inlineStr">
         <is>
-          <t>Confirm the value of password history: Previous passwords refused (local accounts). Delivered: 8 (to be set to 10).</t>
+          <t>Confirm the value of password history: Previous passwords refused (local accounts). Delivered: 10.</t>
         </is>
       </c>
       <c r="F21" s="24" t="inlineStr">
@@ -12288,7 +12394,7 @@
       </c>
       <c r="G21" s="24" t="inlineStr">
         <is>
-          <t>8 (to be set to 10)</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H21" s="24" t="inlineStr">

</xml_diff>